<commit_message>
built factor style but didnt get good feedback, changed data source to adjustment closing price
</commit_message>
<xml_diff>
--- a/D_analysis/check_output/IC_score.xlsx
+++ b/D_analysis/check_output/IC_score.xlsx
@@ -2566,7 +2566,7 @@
         <v>0</v>
       </c>
       <c r="C92">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D92">
         <v>0.5</v>
@@ -2575,7 +2575,7 @@
         <v>0.5</v>
       </c>
       <c r="F92">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="93" spans="1:6">

</xml_diff>